<commit_message>
Actualizacion automatica de Valuacion por Multiplos (2026-09-09)
</commit_message>
<xml_diff>
--- a/data/valuacion_multiplos.xlsx
+++ b/data/valuacion_multiplos.xlsx
@@ -735,10 +735,10 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2465</v>
+        <v>2455</v>
       </c>
       <c r="G3" t="n">
-        <v>4.88</v>
+        <v>4.86</v>
       </c>
       <c r="H3" t="n">
         <v>5.31</v>
@@ -746,7 +746,7 @@
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="n">
-        <v>4</v>
+        <v>3.98</v>
       </c>
       <c r="L3" t="n">
         <v>2.32</v>
@@ -766,7 +766,7 @@
       </c>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="n">
-        <v>14.71</v>
+        <v>14.65</v>
       </c>
       <c r="T3" t="n">
         <v>7.98</v>
@@ -786,25 +786,25 @@
       </c>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="n">
-        <v>2313.33</v>
+        <v>2312.86</v>
       </c>
       <c r="AB3" t="n">
-        <v>2261.96</v>
+        <v>2261.76</v>
       </c>
       <c r="AC3" t="n">
-        <v>1238.81</v>
+        <v>1238.76</v>
       </c>
       <c r="AD3" t="n">
-        <v>-0.008</v>
+        <v>-0.0121</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.1573</v>
+        <v>0.1526</v>
       </c>
       <c r="AF3" t="n">
-        <v>0.5488</v>
+        <v>0.5425</v>
       </c>
       <c r="AG3" t="n">
-        <v>-0.0645</v>
+        <v>-0.0683</v>
       </c>
       <c r="AH3" t="inlineStr"/>
       <c r="AI3" t="n">
@@ -813,9 +813,7 @@
       <c r="AJ3" t="n">
         <v>1</v>
       </c>
-      <c r="AK3" t="n">
-        <v>-0.07630000000000001</v>
-      </c>
+      <c r="AK3" t="inlineStr"/>
       <c r="AL3" t="n">
         <v>1.34</v>
       </c>
@@ -993,7 +991,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2855</v>
+        <v>2867.5</v>
       </c>
       <c r="G5" t="n">
         <v>8.99</v>
@@ -1016,7 +1014,7 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="n">
-        <v>8.48</v>
+        <v>8.52</v>
       </c>
       <c r="T5" t="n">
         <v>40.27</v>
@@ -1030,23 +1028,23 @@
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="n">
-        <v>3012.98</v>
+        <v>3013.57</v>
       </c>
       <c r="AB5" t="n">
-        <v>3000.01</v>
+        <v>3000.26</v>
       </c>
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="n">
-        <v>-0.1154</v>
+        <v>-0.1115</v>
       </c>
       <c r="AE5" t="n">
-        <v>-0.0805</v>
+        <v>-0.0765</v>
       </c>
       <c r="AF5" t="n">
-        <v>0.7825</v>
+        <v>0.7903</v>
       </c>
       <c r="AG5" t="n">
-        <v>-0.1992</v>
+        <v>-0.1957</v>
       </c>
       <c r="AH5" t="inlineStr"/>
       <c r="AI5" t="n">
@@ -1100,7 +1098,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>41.09</v>
+        <v>41.14</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
@@ -1123,7 +1121,7 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="n">
-        <v>19.98</v>
+        <v>20.01</v>
       </c>
       <c r="T6" t="n">
         <v>17.95</v>
@@ -1152,16 +1150,16 @@
         <v>51.61</v>
       </c>
       <c r="AD6" t="n">
-        <v>-0.08649999999999999</v>
+        <v>-0.0854</v>
       </c>
       <c r="AE6" t="n">
-        <v>-0.0221</v>
+        <v>-0.0209</v>
       </c>
       <c r="AF6" t="n">
-        <v>0.2373</v>
+        <v>0.2388</v>
       </c>
       <c r="AG6" t="n">
-        <v>-0.4857</v>
+        <v>-0.4851</v>
       </c>
       <c r="AH6" t="inlineStr"/>
       <c r="AI6" t="n">
@@ -1170,9 +1168,7 @@
       <c r="AJ6" t="n">
         <v>0.75</v>
       </c>
-      <c r="AK6" t="n">
-        <v>-0.1596</v>
-      </c>
+      <c r="AK6" t="inlineStr"/>
       <c r="AL6" t="inlineStr"/>
       <c r="AM6" t="inlineStr">
         <is>
@@ -1217,7 +1213,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>312</v>
+        <v>308.5</v>
       </c>
       <c r="G7" t="n">
         <v>30.61</v>
@@ -1228,7 +1224,7 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
-        <v>0.91</v>
+        <v>0.9</v>
       </c>
       <c r="L7" t="n">
         <v>0.86</v>
@@ -1242,7 +1238,7 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="n">
-        <v>2.94</v>
+        <v>2.91</v>
       </c>
       <c r="T7" t="n">
         <v>4.04</v>
@@ -1250,7 +1246,7 @@
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="X7" t="n">
         <v>0.95</v>
@@ -1260,25 +1256,25 @@
       </c>
       <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="n">
-        <v>326.33</v>
+        <v>326.16</v>
       </c>
       <c r="AB7" t="n">
-        <v>367.26</v>
+        <v>367.19</v>
       </c>
       <c r="AC7" t="n">
-        <v>246.8</v>
+        <v>246.78</v>
       </c>
       <c r="AD7" t="n">
-        <v>-0.1136</v>
+        <v>-0.1236</v>
       </c>
       <c r="AE7" t="n">
-        <v>-0.0951</v>
+        <v>-0.1052</v>
       </c>
       <c r="AF7" t="n">
-        <v>0.5888</v>
+        <v>0.571</v>
       </c>
       <c r="AG7" t="n">
-        <v>-0.4271</v>
+        <v>-0.4336</v>
       </c>
       <c r="AH7" t="inlineStr"/>
       <c r="AI7" t="n">
@@ -1287,9 +1283,7 @@
       <c r="AJ7" t="n">
         <v>1</v>
       </c>
-      <c r="AK7" t="n">
-        <v>-0.0365</v>
-      </c>
+      <c r="AK7" t="inlineStr"/>
       <c r="AL7" t="inlineStr"/>
       <c r="AM7" t="inlineStr">
         <is>
@@ -1465,10 +1459,10 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G9" t="n">
-        <v>13.53</v>
+        <v>13.58</v>
       </c>
       <c r="H9" t="n">
         <v>8.199999999999999</v>
@@ -1478,7 +1472,7 @@
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="n">
-        <v>6.93</v>
+        <v>6.96</v>
       </c>
       <c r="L9" t="n">
         <v>8.33</v>
@@ -1494,7 +1488,7 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="n">
-        <v>8.529999999999999</v>
+        <v>8.56</v>
       </c>
       <c r="T9" t="n">
         <v>6.05</v>
@@ -1502,7 +1496,7 @@
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="n">
-        <v>3</v>
+        <v>3.01</v>
       </c>
       <c r="X9" t="n">
         <v>2.42</v>
@@ -1512,25 +1506,25 @@
       </c>
       <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="n">
-        <v>290.86</v>
+        <v>290.9</v>
       </c>
       <c r="AB9" t="n">
-        <v>292.21</v>
+        <v>292.23</v>
       </c>
       <c r="AC9" t="n">
-        <v>161.96</v>
+        <v>161.97</v>
       </c>
       <c r="AD9" t="n">
-        <v>-0.137</v>
+        <v>-0.1337</v>
       </c>
       <c r="AE9" t="n">
-        <v>-0.1334</v>
+        <v>-0.1301</v>
       </c>
       <c r="AF9" t="n">
-        <v>0.6649</v>
+        <v>0.6712</v>
       </c>
       <c r="AG9" t="n">
-        <v>-0.2219</v>
+        <v>-0.2189</v>
       </c>
       <c r="AH9" t="inlineStr"/>
       <c r="AI9" t="n">
@@ -1539,9 +1533,7 @@
       <c r="AJ9" t="n">
         <v>0.5</v>
       </c>
-      <c r="AK9" t="n">
-        <v>0.6211</v>
-      </c>
+      <c r="AK9" t="inlineStr"/>
       <c r="AL9" t="inlineStr"/>
       <c r="AM9" t="inlineStr">
         <is>
@@ -1586,7 +1578,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>21.85</v>
+        <v>22.1</v>
       </c>
       <c r="G10" t="n">
         <v>91.3</v>
@@ -1623,7 +1615,7 @@
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="n">
-        <v>0.68</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="X10" t="n">
         <v>1.35</v>
@@ -1633,25 +1625,25 @@
       </c>
       <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="n">
-        <v>25.83</v>
+        <v>25.84</v>
       </c>
       <c r="AB10" t="n">
-        <v>31.48</v>
+        <v>31.49</v>
       </c>
       <c r="AC10" t="n">
-        <v>25.86</v>
+        <v>25.87</v>
       </c>
       <c r="AD10" t="n">
-        <v>-0.214</v>
+        <v>-0.205</v>
       </c>
       <c r="AE10" t="n">
-        <v>-0.2491</v>
+        <v>-0.2405</v>
       </c>
       <c r="AF10" t="n">
-        <v>-0.2906</v>
+        <v>-0.2825</v>
       </c>
       <c r="AG10" t="n">
-        <v>-0.5716</v>
+        <v>-0.5667</v>
       </c>
       <c r="AH10" t="inlineStr"/>
       <c r="AI10" t="n">
@@ -1660,9 +1652,7 @@
       <c r="AJ10" t="n">
         <v>0.25</v>
       </c>
-      <c r="AK10" t="n">
-        <v>0.0387</v>
-      </c>
+      <c r="AK10" t="inlineStr"/>
       <c r="AL10" t="n">
         <v>3.01</v>
       </c>
@@ -1909,10 +1899,10 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3105</v>
+        <v>3115</v>
       </c>
       <c r="G13" t="n">
-        <v>5.83</v>
+        <v>5.85</v>
       </c>
       <c r="H13" t="n">
         <v>14.57</v>
@@ -1922,7 +1912,7 @@
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
-        <v>2.08</v>
+        <v>2.09</v>
       </c>
       <c r="L13" t="n">
         <v>1.9</v>
@@ -1942,7 +1932,7 @@
       </c>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="n">
-        <v>10.91</v>
+        <v>10.95</v>
       </c>
       <c r="T13" t="n">
         <v>22.25</v>
@@ -1962,25 +1952,25 @@
       </c>
       <c r="Z13" t="inlineStr"/>
       <c r="AA13" t="n">
-        <v>3152.32</v>
+        <v>3152.8</v>
       </c>
       <c r="AB13" t="n">
-        <v>3051.36</v>
+        <v>3051.56</v>
       </c>
       <c r="AC13" t="n">
-        <v>1501.62</v>
+        <v>1501.67</v>
       </c>
       <c r="AD13" t="n">
-        <v>-0.0806</v>
+        <v>-0.07770000000000001</v>
       </c>
       <c r="AE13" t="n">
-        <v>-0.1296</v>
+        <v>-0.1268</v>
       </c>
       <c r="AF13" t="n">
-        <v>0.927</v>
+        <v>0.9332</v>
       </c>
       <c r="AG13" t="n">
-        <v>-0.1488</v>
+        <v>-0.1461</v>
       </c>
       <c r="AH13" t="inlineStr"/>
       <c r="AI13" t="n">
@@ -1989,9 +1979,7 @@
       <c r="AJ13" t="n">
         <v>1</v>
       </c>
-      <c r="AK13" t="n">
-        <v>0.285</v>
-      </c>
+      <c r="AK13" t="inlineStr"/>
       <c r="AL13" t="n">
         <v>-0.21</v>
       </c>
@@ -2100,9 +2088,7 @@
       <c r="AJ14" t="n">
         <v>0.5</v>
       </c>
-      <c r="AK14" t="n">
-        <v>-0.134</v>
-      </c>
+      <c r="AK14" t="inlineStr"/>
       <c r="AL14" t="inlineStr"/>
       <c r="AM14" t="inlineStr">
         <is>
@@ -2248,10 +2234,10 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>540.5</v>
+        <v>547.5</v>
       </c>
       <c r="G16" t="n">
-        <v>10.76</v>
+        <v>10.9</v>
       </c>
       <c r="H16" t="n">
         <v>11.33</v>
@@ -2261,7 +2247,7 @@
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="n">
-        <v>2.28</v>
+        <v>2.31</v>
       </c>
       <c r="L16" t="n">
         <v>0.79</v>
@@ -2281,7 +2267,7 @@
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="n">
-        <v>1.37</v>
+        <v>1.39</v>
       </c>
       <c r="X16" t="n">
         <v>1.5</v>
@@ -2291,25 +2277,25 @@
       </c>
       <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="n">
-        <v>623.13</v>
+        <v>623.47</v>
       </c>
       <c r="AB16" t="n">
-        <v>558.85</v>
+        <v>558.99</v>
       </c>
       <c r="AC16" t="n">
-        <v>311.04</v>
+        <v>311.07</v>
       </c>
       <c r="AD16" t="n">
-        <v>-0.1322</v>
+        <v>-0.121</v>
       </c>
       <c r="AE16" t="n">
-        <v>-0.0898</v>
+        <v>-0.078</v>
       </c>
       <c r="AF16" t="n">
-        <v>1.0183</v>
+        <v>1.0444</v>
       </c>
       <c r="AG16" t="n">
-        <v>-0.2506</v>
+        <v>-0.2409</v>
       </c>
       <c r="AH16" t="inlineStr"/>
       <c r="AI16" t="n">
@@ -2318,9 +2304,7 @@
       <c r="AJ16" t="n">
         <v>0.75</v>
       </c>
-      <c r="AK16" t="n">
-        <v>0.1226</v>
-      </c>
+      <c r="AK16" t="inlineStr"/>
       <c r="AL16" t="n">
         <v>-4.34</v>
       </c>
@@ -2492,7 +2476,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -2529,25 +2513,25 @@
       </c>
       <c r="Z18" t="inlineStr"/>
       <c r="AA18" t="n">
-        <v>434.14</v>
+        <v>434.05</v>
       </c>
       <c r="AB18" t="n">
-        <v>471.91</v>
+        <v>471.87</v>
       </c>
       <c r="AC18" t="n">
-        <v>341.65</v>
+        <v>341.64</v>
       </c>
       <c r="AD18" t="n">
-        <v>-0.0386</v>
+        <v>-0.0432</v>
       </c>
       <c r="AE18" t="n">
-        <v>-0.1523</v>
+        <v>-0.1563</v>
       </c>
       <c r="AF18" t="n">
-        <v>0.5216</v>
+        <v>0.5144</v>
       </c>
       <c r="AG18" t="n">
-        <v>-0.3502</v>
+        <v>-0.3533</v>
       </c>
       <c r="AH18" t="inlineStr"/>
       <c r="AI18" t="n">
@@ -2556,9 +2540,7 @@
       <c r="AJ18" t="n">
         <v>0.333</v>
       </c>
-      <c r="AK18" t="n">
-        <v>0.1965</v>
-      </c>
+      <c r="AK18" t="inlineStr"/>
       <c r="AL18" t="n">
         <v>0.42</v>
       </c>
@@ -2827,76 +2809,78 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>882</v>
+        <v>888.5</v>
       </c>
       <c r="G21" t="n">
-        <v>9.550000000000001</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>10.56</v>
+        <v>76.51000000000001</v>
       </c>
       <c r="I21" t="n">
-        <v>8.199999999999999</v>
+        <v>58.4</v>
       </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="n">
-        <v>1.25</v>
+        <v>1.26</v>
       </c>
       <c r="L21" t="n">
-        <v>1.28</v>
+        <v>1.21</v>
       </c>
       <c r="M21" t="n">
-        <v>1.11</v>
+        <v>1.12</v>
       </c>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="n">
         <v>10.09</v>
       </c>
       <c r="P21" t="n">
-        <v>8.08</v>
+        <v>8.26</v>
       </c>
       <c r="Q21" t="n">
-        <v>6.49</v>
+        <v>7.04</v>
       </c>
       <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
+      <c r="S21" t="n">
+        <v>4.96</v>
+      </c>
       <c r="T21" t="n">
-        <v>20.23</v>
+        <v>17.18</v>
       </c>
       <c r="U21" t="n">
-        <v>15.14</v>
+        <v>15.33</v>
       </c>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="n">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
       <c r="X21" t="n">
-        <v>1.42</v>
+        <v>1.36</v>
       </c>
       <c r="Y21" t="n">
         <v>1.29</v>
       </c>
       <c r="Z21" t="inlineStr"/>
       <c r="AA21" t="n">
-        <v>947.6900000000001</v>
+        <v>948</v>
       </c>
       <c r="AB21" t="n">
-        <v>944.37</v>
+        <v>944.5</v>
       </c>
       <c r="AC21" t="n">
-        <v>758.72</v>
+        <v>758.75</v>
       </c>
       <c r="AD21" t="n">
-        <v>-0.1429</v>
+        <v>-0.1365</v>
       </c>
       <c r="AE21" t="n">
-        <v>0.115</v>
+        <v>0.1233</v>
       </c>
       <c r="AF21" t="n">
-        <v>0.3283</v>
+        <v>0.3381</v>
       </c>
       <c r="AG21" t="n">
-        <v>-0.2109</v>
+        <v>-0.205</v>
       </c>
       <c r="AH21" t="inlineStr"/>
       <c r="AI21" t="n">
@@ -2905,11 +2889,9 @@
       <c r="AJ21" t="n">
         <v>0.75</v>
       </c>
-      <c r="AK21" t="n">
-        <v>-0.1662</v>
-      </c>
+      <c r="AK21" t="inlineStr"/>
       <c r="AL21" t="n">
-        <v>3.33</v>
+        <v>1.01</v>
       </c>
       <c r="AM21" t="inlineStr">
         <is>
@@ -3309,14 +3291,14 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>456</v>
+        <v>450</v>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="n">
-        <v>4.64</v>
+        <v>4.58</v>
       </c>
       <c r="L25" t="n">
         <v>16.69</v>
@@ -3332,13 +3314,13 @@
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="n">
-        <v>58.28</v>
+        <v>57.51</v>
       </c>
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr"/>
       <c r="W25" t="n">
-        <v>13.42</v>
+        <v>13.25</v>
       </c>
       <c r="X25" t="n">
         <v>28.92</v>
@@ -3348,25 +3330,25 @@
       </c>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="n">
-        <v>501.1</v>
+        <v>500.81</v>
       </c>
       <c r="AB25" t="n">
-        <v>572.3200000000001</v>
+        <v>572.2</v>
       </c>
       <c r="AC25" t="n">
-        <v>649.79</v>
+        <v>649.76</v>
       </c>
       <c r="AD25" t="n">
-        <v>-0.0898</v>
+        <v>-0.1018</v>
       </c>
       <c r="AE25" t="n">
-        <v>-0.1739</v>
+        <v>-0.1848</v>
       </c>
       <c r="AF25" t="n">
-        <v>0.2095</v>
+        <v>0.1936</v>
       </c>
       <c r="AG25" t="n">
-        <v>-0.4847</v>
+        <v>-0.4915</v>
       </c>
       <c r="AH25" t="inlineStr"/>
       <c r="AI25" t="n">
@@ -3375,9 +3357,7 @@
       <c r="AJ25" t="n">
         <v>0.25</v>
       </c>
-      <c r="AK25" t="n">
-        <v>0.476</v>
-      </c>
+      <c r="AK25" t="inlineStr"/>
       <c r="AL25" t="n">
         <v>16.78</v>
       </c>
@@ -3555,10 +3535,10 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>3247.5</v>
+        <v>3235</v>
       </c>
       <c r="G27" t="n">
-        <v>7.31</v>
+        <v>7.28</v>
       </c>
       <c r="H27" t="n">
         <v>15.76</v>
@@ -3568,7 +3548,7 @@
       </c>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="n">
-        <v>2.37</v>
+        <v>2.36</v>
       </c>
       <c r="L27" t="n">
         <v>3.28</v>
@@ -3588,13 +3568,13 @@
       </c>
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="n">
-        <v>4.01</v>
+        <v>4</v>
       </c>
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="n">
-        <v>1.1</v>
+        <v>1.09</v>
       </c>
       <c r="X27" t="n">
         <v>1.41</v>
@@ -3604,25 +3584,25 @@
       </c>
       <c r="Z27" t="inlineStr"/>
       <c r="AA27" t="n">
-        <v>3702.56</v>
+        <v>3701.96</v>
       </c>
       <c r="AB27" t="n">
-        <v>3834.1</v>
+        <v>3833.85</v>
       </c>
       <c r="AC27" t="n">
-        <v>2266.2</v>
+        <v>2266.14</v>
       </c>
       <c r="AD27" t="n">
-        <v>-0.2055</v>
+        <v>-0.2085</v>
       </c>
       <c r="AE27" t="n">
-        <v>-0.243</v>
+        <v>-0.2459</v>
       </c>
       <c r="AF27" t="n">
-        <v>0.2994</v>
+        <v>0.2944</v>
       </c>
       <c r="AG27" t="n">
-        <v>-0.3201</v>
+        <v>-0.3227</v>
       </c>
       <c r="AH27" t="inlineStr"/>
       <c r="AI27" t="n">
@@ -3631,9 +3611,7 @@
       <c r="AJ27" t="n">
         <v>0.5</v>
       </c>
-      <c r="AK27" t="n">
-        <v>0.5399</v>
-      </c>
+      <c r="AK27" t="inlineStr"/>
       <c r="AL27" t="n">
         <v>0.02</v>
       </c>
@@ -3811,7 +3789,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>822.5</v>
+        <v>827.5</v>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
@@ -3838,7 +3816,7 @@
       </c>
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="n">
-        <v>12.24</v>
+        <v>12.32</v>
       </c>
       <c r="T29" t="n">
         <v>8.779999999999999</v>
@@ -3856,25 +3834,25 @@
       </c>
       <c r="Z29" t="inlineStr"/>
       <c r="AA29" t="n">
-        <v>771.05</v>
+        <v>771.29</v>
       </c>
       <c r="AB29" t="n">
-        <v>847.12</v>
+        <v>847.22</v>
       </c>
       <c r="AC29" t="n">
-        <v>811.6799999999999</v>
+        <v>811.7</v>
       </c>
       <c r="AD29" t="n">
-        <v>0.0808</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="AE29" t="n">
-        <v>0.113</v>
+        <v>0.1198</v>
       </c>
       <c r="AF29" t="n">
-        <v>-0.09619999999999999</v>
+        <v>-0.0907</v>
       </c>
       <c r="AG29" t="n">
-        <v>-0.2689</v>
+        <v>-0.2644</v>
       </c>
       <c r="AH29" t="inlineStr"/>
       <c r="AI29" t="n">
@@ -3883,9 +3861,7 @@
       <c r="AJ29" t="n">
         <v>0.75</v>
       </c>
-      <c r="AK29" t="n">
-        <v>-0.09429999999999999</v>
-      </c>
+      <c r="AK29" t="inlineStr"/>
       <c r="AL29" t="n">
         <v>2.71</v>
       </c>
@@ -4620,85 +4596,87 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>1225</v>
+        <v>1250</v>
       </c>
       <c r="G36" t="n">
-        <v>23.32</v>
+        <v>23.79</v>
       </c>
       <c r="H36" t="n">
-        <v>7.34</v>
+        <v>16.98</v>
       </c>
       <c r="I36" t="n">
-        <v>5.76</v>
+        <v>13.71</v>
       </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="n">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="L36" t="n">
-        <v>0.2</v>
+        <v>0.23</v>
       </c>
       <c r="M36" t="n">
-        <v>0.2</v>
+        <v>0.18</v>
       </c>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="n">
         <v>26.06</v>
       </c>
       <c r="P36" t="n">
-        <v>4.2</v>
+        <v>5.69</v>
       </c>
       <c r="Q36" t="n">
-        <v>3.69</v>
+        <v>4.67</v>
       </c>
       <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
-      <c r="T36" t="inlineStr"/>
+      <c r="S36" t="n">
+        <v>8.01</v>
+      </c>
+      <c r="T36" t="n">
+        <v>10.34</v>
+      </c>
       <c r="U36" t="inlineStr"/>
       <c r="V36" t="inlineStr"/>
       <c r="W36" t="n">
-        <v>0.84</v>
+        <v>0.86</v>
       </c>
       <c r="X36" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.02</v>
       </c>
       <c r="Y36" t="n">
-        <v>0.76</v>
+        <v>0.85</v>
       </c>
       <c r="Z36" t="inlineStr"/>
       <c r="AA36" t="n">
-        <v>1269.76</v>
+        <v>1270.95</v>
       </c>
       <c r="AB36" t="n">
-        <v>1311.47</v>
+        <v>1311.97</v>
       </c>
       <c r="AC36" t="n">
-        <v>990.3200000000001</v>
+        <v>990.45</v>
       </c>
       <c r="AD36" t="n">
-        <v>-0.1026</v>
+        <v>-0.0842</v>
       </c>
       <c r="AE36" t="n">
-        <v>0.0251</v>
+        <v>0.046</v>
       </c>
       <c r="AF36" t="n">
-        <v>0.162</v>
+        <v>0.1857</v>
       </c>
       <c r="AG36" t="n">
-        <v>-0.2857</v>
+        <v>-0.2711</v>
       </c>
       <c r="AH36" t="inlineStr"/>
       <c r="AI36" t="n">
         <v>1</v>
       </c>
       <c r="AJ36" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AK36" t="n">
-        <v>0.0131</v>
-      </c>
+        <v>0.75</v>
+      </c>
+      <c r="AK36" t="inlineStr"/>
       <c r="AL36" t="n">
-        <v>1.1</v>
+        <v>0.58</v>
       </c>
       <c r="AM36" t="inlineStr">
         <is>
@@ -4834,7 +4812,7 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>2930</v>
+        <v>3020</v>
       </c>
       <c r="G38" t="n">
         <v>21.88</v>
@@ -4847,7 +4825,7 @@
       </c>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="n">
-        <v>2.99</v>
+        <v>3.08</v>
       </c>
       <c r="L38" t="n">
         <v>2.67</v>
@@ -4865,7 +4843,7 @@
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="n">
-        <v>14.87</v>
+        <v>15.33</v>
       </c>
       <c r="T38" t="n">
         <v>15.85</v>
@@ -4873,7 +4851,7 @@
       <c r="U38" t="inlineStr"/>
       <c r="V38" t="inlineStr"/>
       <c r="W38" t="n">
-        <v>0.93</v>
+        <v>0.96</v>
       </c>
       <c r="X38" t="n">
         <v>0.6899999999999999</v>
@@ -4883,22 +4861,22 @@
       </c>
       <c r="Z38" t="inlineStr"/>
       <c r="AA38" t="n">
-        <v>2249.05</v>
+        <v>2253.33</v>
       </c>
       <c r="AB38" t="n">
-        <v>2150.01</v>
+        <v>2151.81</v>
       </c>
       <c r="AC38" t="n">
-        <v>1282.91</v>
+        <v>1283.36</v>
       </c>
       <c r="AD38" t="n">
-        <v>0.3228</v>
+        <v>0.3634</v>
       </c>
       <c r="AE38" t="n">
-        <v>0.3998</v>
+        <v>0.4428</v>
       </c>
       <c r="AF38" t="n">
-        <v>0.4759</v>
+        <v>0.5212</v>
       </c>
       <c r="AG38" t="n">
         <v>0</v>
@@ -4910,9 +4888,7 @@
       <c r="AJ38" t="n">
         <v>0.75</v>
       </c>
-      <c r="AK38" t="n">
-        <v>-0.0172</v>
-      </c>
+      <c r="AK38" t="inlineStr"/>
       <c r="AL38" t="n">
         <v>-3.21</v>
       </c>
@@ -5357,10 +5333,10 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>2341</v>
+        <v>2344</v>
       </c>
       <c r="G43" t="n">
-        <v>10.29</v>
+        <v>10.3</v>
       </c>
       <c r="H43" t="n">
         <v>6.46</v>
@@ -5390,7 +5366,7 @@
       </c>
       <c r="R43" t="inlineStr"/>
       <c r="S43" t="n">
-        <v>36.74</v>
+        <v>36.79</v>
       </c>
       <c r="T43" t="n">
         <v>16.25</v>
@@ -5410,25 +5386,25 @@
       </c>
       <c r="Z43" t="inlineStr"/>
       <c r="AA43" t="n">
-        <v>1931.08</v>
+        <v>1931.22</v>
       </c>
       <c r="AB43" t="n">
-        <v>1958.04</v>
+        <v>1958.1</v>
       </c>
       <c r="AC43" t="n">
-        <v>1209.74</v>
+        <v>1209.75</v>
       </c>
       <c r="AD43" t="n">
-        <v>0.3037</v>
+        <v>0.3054</v>
       </c>
       <c r="AE43" t="n">
-        <v>0.3011</v>
+        <v>0.3027</v>
       </c>
       <c r="AF43" t="n">
-        <v>1.0224</v>
+        <v>1.025</v>
       </c>
       <c r="AG43" t="n">
-        <v>-0.0563</v>
+        <v>-0.0551</v>
       </c>
       <c r="AH43" t="inlineStr"/>
       <c r="AI43" t="n">
@@ -5437,9 +5413,7 @@
       <c r="AJ43" t="n">
         <v>1</v>
       </c>
-      <c r="AK43" t="n">
-        <v>0.0544</v>
-      </c>
+      <c r="AK43" t="inlineStr"/>
       <c r="AL43" t="n">
         <v>-0.1</v>
       </c>
@@ -5486,10 +5460,10 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>1760</v>
+        <v>1755</v>
       </c>
       <c r="G44" t="n">
-        <v>3.53</v>
+        <v>3.52</v>
       </c>
       <c r="H44" t="n">
         <v>5.05</v>
@@ -5519,7 +5493,7 @@
       </c>
       <c r="R44" t="inlineStr"/>
       <c r="S44" t="n">
-        <v>5.03</v>
+        <v>5.02</v>
       </c>
       <c r="T44" t="n">
         <v>4.13</v>
@@ -5539,25 +5513,25 @@
       </c>
       <c r="Z44" t="inlineStr"/>
       <c r="AA44" t="n">
-        <v>1688.71</v>
+        <v>1688.47</v>
       </c>
       <c r="AB44" t="n">
-        <v>1642.32</v>
+        <v>1642.22</v>
       </c>
       <c r="AC44" t="n">
-        <v>946.21</v>
+        <v>946.1900000000001</v>
       </c>
       <c r="AD44" t="n">
-        <v>0.1279</v>
+        <v>0.1247</v>
       </c>
       <c r="AE44" t="n">
-        <v>0.1161</v>
+        <v>0.113</v>
       </c>
       <c r="AF44" t="n">
-        <v>0.7477</v>
+        <v>0.7428</v>
       </c>
       <c r="AG44" t="n">
-        <v>-0.111</v>
+        <v>-0.1135</v>
       </c>
       <c r="AH44" t="inlineStr"/>
       <c r="AI44" t="n">
@@ -5566,9 +5540,7 @@
       <c r="AJ44" t="n">
         <v>1</v>
       </c>
-      <c r="AK44" t="n">
-        <v>0.1313</v>
-      </c>
+      <c r="AK44" t="inlineStr"/>
       <c r="AL44" t="n">
         <v>-0.3</v>
       </c>
@@ -5960,14 +5932,14 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>1780</v>
+        <v>1790</v>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="n">
-        <v>2.18</v>
+        <v>2.19</v>
       </c>
       <c r="L48" t="n">
         <v>4.08</v>
@@ -5989,7 +5961,7 @@
       </c>
       <c r="V48" t="inlineStr"/>
       <c r="W48" t="n">
-        <v>0.77</v>
+        <v>0.78</v>
       </c>
       <c r="X48" t="n">
         <v>0.98</v>
@@ -5999,25 +5971,25 @@
       </c>
       <c r="Z48" t="inlineStr"/>
       <c r="AA48" t="n">
-        <v>1897.85</v>
+        <v>1898.33</v>
       </c>
       <c r="AB48" t="n">
-        <v>2001.78</v>
+        <v>2001.98</v>
       </c>
       <c r="AC48" t="n">
-        <v>1587.83</v>
+        <v>1587.88</v>
       </c>
       <c r="AD48" t="n">
-        <v>-0.07049999999999999</v>
+        <v>-0.0653</v>
       </c>
       <c r="AE48" t="n">
-        <v>-0.0404</v>
+        <v>-0.035</v>
       </c>
       <c r="AF48" t="n">
-        <v>0.1447</v>
+        <v>0.1511</v>
       </c>
       <c r="AG48" t="n">
-        <v>-0.2675</v>
+        <v>-0.2634</v>
       </c>
       <c r="AH48" t="inlineStr"/>
       <c r="AI48" t="n">
@@ -6026,9 +5998,7 @@
       <c r="AJ48" t="n">
         <v>0.75</v>
       </c>
-      <c r="AK48" t="n">
-        <v>-0.0555</v>
-      </c>
+      <c r="AK48" t="inlineStr"/>
       <c r="AL48" t="n">
         <v>-4.74</v>
       </c>
@@ -6347,9 +6317,7 @@
       <c r="AJ51" t="n">
         <v>0.75</v>
       </c>
-      <c r="AK51" t="n">
-        <v>-0.0446</v>
-      </c>
+      <c r="AK51" t="inlineStr"/>
       <c r="AL51" t="n">
         <v>1.56</v>
       </c>
@@ -6600,10 +6568,10 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>1575</v>
+        <v>1565</v>
       </c>
       <c r="G54" t="n">
-        <v>6.38</v>
+        <v>6.34</v>
       </c>
       <c r="H54" t="n">
         <v>10.77</v>
@@ -6633,7 +6601,7 @@
       </c>
       <c r="R54" t="inlineStr"/>
       <c r="S54" t="n">
-        <v>9.48</v>
+        <v>9.42</v>
       </c>
       <c r="T54" t="n">
         <v>10.7</v>
@@ -6641,7 +6609,7 @@
       <c r="U54" t="inlineStr"/>
       <c r="V54" t="inlineStr"/>
       <c r="W54" t="n">
-        <v>1.2</v>
+        <v>1.19</v>
       </c>
       <c r="X54" t="n">
         <v>1.39</v>
@@ -6651,25 +6619,25 @@
       </c>
       <c r="Z54" t="inlineStr"/>
       <c r="AA54" t="n">
-        <v>1622.6</v>
+        <v>1622.13</v>
       </c>
       <c r="AB54" t="n">
-        <v>1708.08</v>
+        <v>1707.88</v>
       </c>
       <c r="AC54" t="n">
-        <v>1060.75</v>
+        <v>1060.7</v>
       </c>
       <c r="AD54" t="n">
-        <v>-0.0247</v>
+        <v>-0.0309</v>
       </c>
       <c r="AE54" t="n">
-        <v>-0.1051</v>
+        <v>-0.1108</v>
       </c>
       <c r="AF54" t="n">
-        <v>0.497</v>
+        <v>0.4875</v>
       </c>
       <c r="AG54" t="n">
-        <v>-0.2775</v>
+        <v>-0.2821</v>
       </c>
       <c r="AH54" t="inlineStr"/>
       <c r="AI54" t="n">
@@ -6678,9 +6646,7 @@
       <c r="AJ54" t="n">
         <v>0.5</v>
       </c>
-      <c r="AK54" t="n">
-        <v>0.1998</v>
-      </c>
+      <c r="AK54" t="inlineStr"/>
       <c r="AL54" t="inlineStr"/>
       <c r="AM54" t="inlineStr">
         <is>
@@ -29983,10 +29949,10 @@
         </is>
       </c>
       <c r="F259" t="n">
-        <v>1910</v>
+        <v>1920</v>
       </c>
       <c r="G259" t="n">
-        <v>115.76</v>
+        <v>116.36</v>
       </c>
       <c r="H259" t="inlineStr"/>
       <c r="I259" t="inlineStr"/>
@@ -30014,7 +29980,7 @@
       <c r="U259" t="inlineStr"/>
       <c r="V259" t="inlineStr"/>
       <c r="W259" t="n">
-        <v>0.7</v>
+        <v>0.71</v>
       </c>
       <c r="X259" t="n">
         <v>5.03</v>
@@ -30024,25 +29990,25 @@
       </c>
       <c r="Z259" t="inlineStr"/>
       <c r="AA259" t="n">
-        <v>12761.67</v>
+        <v>12762.14</v>
       </c>
       <c r="AB259" t="n">
-        <v>17731.84</v>
+        <v>17732.04</v>
       </c>
       <c r="AC259" t="n">
-        <v>15997.18</v>
+        <v>15997.23</v>
       </c>
       <c r="AD259" t="n">
-        <v>-0.8885999999999999</v>
+        <v>-0.888</v>
       </c>
       <c r="AE259" t="n">
-        <v>-0.8963</v>
+        <v>-0.8958</v>
       </c>
       <c r="AF259" t="n">
-        <v>-0.8871</v>
+        <v>-0.8866000000000001</v>
       </c>
       <c r="AG259" t="n">
-        <v>-0.9308</v>
+        <v>-0.9304</v>
       </c>
       <c r="AH259" t="inlineStr"/>
       <c r="AI259" t="n">
@@ -30051,9 +30017,7 @@
       <c r="AJ259" t="n">
         <v>0.5</v>
       </c>
-      <c r="AK259" t="n">
-        <v>-0.0217</v>
-      </c>
+      <c r="AK259" t="inlineStr"/>
       <c r="AL259" t="n">
         <v>4.29</v>
       </c>
@@ -31954,10 +31918,10 @@
         </is>
       </c>
       <c r="F276" t="n">
-        <v>23800</v>
+        <v>23825</v>
       </c>
       <c r="G276" t="n">
-        <v>5.2</v>
+        <v>5.21</v>
       </c>
       <c r="H276" t="n">
         <v>9.109999999999999</v>
@@ -31987,7 +31951,7 @@
       </c>
       <c r="R276" t="inlineStr"/>
       <c r="S276" t="n">
-        <v>9.34</v>
+        <v>9.35</v>
       </c>
       <c r="T276" t="n">
         <v>8.609999999999999</v>
@@ -32007,25 +31971,25 @@
       </c>
       <c r="Z276" t="inlineStr"/>
       <c r="AA276" t="n">
-        <v>22875</v>
+        <v>22876.19</v>
       </c>
       <c r="AB276" t="n">
-        <v>23859.85</v>
+        <v>23860.35</v>
       </c>
       <c r="AC276" t="n">
-        <v>16051.06</v>
+        <v>16051.18</v>
       </c>
       <c r="AD276" t="n">
-        <v>0.0248</v>
+        <v>0.0258</v>
       </c>
       <c r="AE276" t="n">
-        <v>-0.0775</v>
+        <v>-0.0766</v>
       </c>
       <c r="AF276" t="n">
-        <v>0.3964</v>
+        <v>0.3978</v>
       </c>
       <c r="AG276" t="n">
-        <v>-0.1185</v>
+        <v>-0.1176</v>
       </c>
       <c r="AH276" t="inlineStr"/>
       <c r="AI276" t="n">
@@ -32034,9 +31998,7 @@
       <c r="AJ276" t="n">
         <v>0.75</v>
       </c>
-      <c r="AK276" t="n">
-        <v>0.0375</v>
-      </c>
+      <c r="AK276" t="inlineStr"/>
       <c r="AL276" t="n">
         <v>0.44</v>
       </c>

</xml_diff>